<commit_message>
Delete slide files, modify setup and readme.
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zlu/Code/UAV/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0BD0F05-662F-0042-BCCD-256A58F8C646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="20040" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
-  <si>
-    <t>Drone</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
   <si>
     <t>基础套件</t>
   </si>
@@ -40,9 +46,6 @@
     <t>电池</t>
   </si>
   <si>
-    <t>格氏6S 4000mAh 30C</t>
-  </si>
-  <si>
     <t>飞塔</t>
   </si>
   <si>
@@ -73,25 +76,64 @@
     <t>机载电脑</t>
   </si>
   <si>
-    <t>Intel NUC11TNKi5</t>
-  </si>
-  <si>
-    <t>19V稳压模块</t>
-  </si>
-  <si>
     <t>3D打印</t>
   </si>
   <si>
     <t>雷达保护罩</t>
+  </si>
+  <si>
+    <t>Intel NUC11TNKv5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>格氏6S 4000mAh 30C / DualSky 3300mAh 50C</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Drone1 - SUPER</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Drone2 - UniQuad250L</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>轴距250mm QAV250机架</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>T-Motor F60 KV1750</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>51466 / 51477</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DualSky 3300mAh 50C</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>19V Buck</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jetson Orin NX 16GB + Damiao board</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>脚架</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>增高角垫</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="0" formatCode="General"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -99,14 +141,17 @@
       <name val="等线"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="FangSong"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color indexed="8"/>
-      <name val="Helvetica Neue"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -178,57 +223,128 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+  <cellXfs count="12">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
   <colors>
     <indexedColors>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
-      <rgbColor rgb="ffff0000"/>
-      <rgbColor rgb="ff00ff00"/>
-      <rgbColor rgb="ff0000ff"/>
-      <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffff00ff"/>
-      <rgbColor rgb="ff00ffff"/>
-      <rgbColor rgb="ff000000"/>
-      <rgbColor rgb="ffffffff"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office Theme">
       <a:dk1>
@@ -430,7 +546,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -448,7 +564,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -477,7 +593,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -502,7 +618,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -527,7 +643,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -552,7 +668,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -577,7 +693,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -602,7 +718,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -627,7 +743,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -652,7 +768,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -677,7 +793,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -690,9 +806,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:spDef>
@@ -709,7 +831,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="91439" tIns="45719" rIns="91439" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:noAutofit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -727,7 +849,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -752,7 +874,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -777,7 +899,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -802,7 +924,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -827,7 +949,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -852,7 +974,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -877,7 +999,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -902,7 +1024,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -927,7 +1049,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -952,7 +1074,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -965,9 +1087,15 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:lnDef>
@@ -981,7 +1109,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -999,7 +1127,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1100" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1028,7 +1156,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1053,7 +1181,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1078,7 +1206,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1103,7 +1231,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1128,7 +1256,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1153,7 +1281,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1178,7 +1306,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1203,7 +1331,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1228,7 +1356,7 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1800" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr kumimoji="0" sz="1800" b="0" i="0" u="none" strike="noStrike" cap="none" spc="0" normalizeH="0" baseline="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
@@ -1241,143 +1369,251 @@
         </a:lvl9pPr>
       </a:lstStyle>
       <a:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
         <a:fontRef idx="none"/>
       </a:style>
     </a:txDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="14.25" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.6719" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col min="3" max="3" width="41" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="32.33203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" spans="1:6" ht="15" customHeight="1" thickBot="1">
+      <c r="A1" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+    </row>
+    <row r="2" spans="1:6" ht="16.5" customHeight="1">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1">
-      <c r="A2" t="s" s="4">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s" s="4">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s" s="4">
+    <row r="3" spans="1:6" ht="16" customHeight="1">
+      <c r="A3" s="7"/>
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
+      <c r="C3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="5"/>
-      <c r="B3" t="s" s="6">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s" s="6">
+    <row r="4" spans="1:6" ht="16" customHeight="1">
+      <c r="A4" s="7"/>
+      <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
+      <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" t="s" s="6">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s" s="6">
+    <row r="5" spans="1:6" ht="16" customHeight="1">
+      <c r="A5" s="7"/>
+      <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="C5" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="5"/>
-      <c r="B5" t="s" s="6">
+    <row r="6" spans="1:6" ht="16" customHeight="1">
+      <c r="A6" s="7"/>
+      <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C5" t="s" s="6">
+      <c r="C6" s="5" t="s">
         <v>9</v>
       </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="5"/>
-      <c r="B6" t="s" s="6">
+    <row r="7" spans="1:6" ht="16" customHeight="1">
+      <c r="A7" s="7"/>
+      <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s" s="6">
+      <c r="C7" s="5" t="s">
         <v>11</v>
       </c>
+      <c r="D7" s="7"/>
+      <c r="E7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" t="s" s="6">
+    <row r="8" spans="1:6" ht="15" customHeight="1" thickBot="1">
+      <c r="A8" s="8"/>
+      <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C7" t="s" s="6">
+      <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" t="s" s="2">
+    <row r="9" spans="1:6" ht="16.5" customHeight="1">
+      <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C8" t="s" s="2">
+      <c r="B9" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" t="s" s="4">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s" s="4">
+    <row r="10" spans="1:6" ht="16" customHeight="1">
+      <c r="A10" s="7"/>
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C9" t="s" s="4">
+      <c r="C10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15" customHeight="1">
+      <c r="A11" s="7"/>
+      <c r="B11" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" ht="16" customHeight="1">
+      <c r="A12" s="5" t="s">
         <v>18</v>
       </c>
+      <c r="B12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="4"/>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="5"/>
-      <c r="B10" t="s" s="6">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s" s="6">
-        <v>20</v>
-      </c>
+    <row r="13" spans="1:6" ht="14.25" customHeight="1">
+      <c r="E13" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="4"/>
     </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" t="s" s="6">
-        <v>21</v>
-      </c>
-      <c r="C11" s="5"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" t="s" s="6">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s" s="6">
-        <v>23</v>
-      </c>
-      <c r="C12" s="5"/>
+    <row r="14" spans="1:6" ht="14.25" customHeight="1">
+      <c r="E14" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
     <mergeCell ref="A2:A8"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D2:D8"/>
+    <mergeCell ref="D9:D11"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;11&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Tested controller on real drone.
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zlu/Code/UAV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0BD0F05-662F-0042-BCCD-256A58F8C646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87BACD13-41E4-8D47-827B-8362B36BDDDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="20040" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>基础套件</t>
   </si>
@@ -47,9 +47,6 @@
   </si>
   <si>
     <t>飞塔</t>
-  </si>
-  <si>
-    <t>NXTPX4v2 + 50A四合一电调</t>
   </si>
   <si>
     <t>接收机</t>
@@ -106,10 +103,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>51466 / 51477</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>DualSky 3300mAh 50C</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -127,6 +120,18 @@
   </si>
   <si>
     <t>增高角垫</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>5寸 51466 / 51477</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NxtPX4v2 + 微空50A四合一电调</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>乐迪R12DSE 2.4G 12通道</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -240,6 +245,12 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -249,13 +260,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1394,26 +1399,26 @@
     <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
     <col min="3" max="3" width="41" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1640625" style="1" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="32.33203125" style="1" customWidth="1"/>
     <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" thickBot="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
     </row>
     <row r="2" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1422,183 +1427,183 @@
       <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="11" t="s">
-        <v>24</v>
+      <c r="F2" s="7" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16" customHeight="1">
-      <c r="A3" s="7"/>
+      <c r="A3" s="9"/>
       <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="7"/>
+      <c r="D3" s="9"/>
       <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>25</v>
+      <c r="F3" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="16" customHeight="1">
-      <c r="A4" s="7"/>
+      <c r="A4" s="9"/>
       <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="9"/>
       <c r="E4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="9" t="s">
-        <v>26</v>
+      <c r="F4" s="6" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16" customHeight="1">
-      <c r="A5" s="7"/>
+      <c r="A5" s="9"/>
       <c r="B5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="7"/>
+      <c r="C5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="9"/>
       <c r="E5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>27</v>
+      <c r="F5" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16" customHeight="1">
-      <c r="A6" s="7"/>
+      <c r="A6" s="9"/>
       <c r="B6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="7"/>
+      <c r="C6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="9"/>
       <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>9</v>
+      <c r="F6" s="6" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="16" customHeight="1">
-      <c r="A7" s="7"/>
+      <c r="A7" s="9"/>
       <c r="B7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="7"/>
+      <c r="D7" s="9"/>
       <c r="E7" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" thickBot="1">
-      <c r="A8" s="8"/>
+      <c r="A8" s="10"/>
       <c r="B8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="8"/>
+      <c r="D8" s="10"/>
       <c r="E8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" customHeight="1">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="16" customHeight="1">
-      <c r="A10" s="7"/>
+      <c r="A10" s="9"/>
       <c r="B10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="7"/>
+        <v>16</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="9"/>
       <c r="E10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>29</v>
+        <v>16</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="7"/>
-      <c r="B11" s="9" t="s">
-        <v>28</v>
+      <c r="A11" s="9"/>
+      <c r="B11" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="C11" s="4"/>
-      <c r="D11" s="7"/>
+      <c r="D11" s="9"/>
       <c r="E11" s="5"/>
       <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6" ht="16" customHeight="1">
       <c r="A12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>19</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>19</v>
       </c>
       <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:6" ht="14.25" customHeight="1">
-      <c r="E13" s="9" t="s">
-        <v>30</v>
+      <c r="E13" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" ht="14.25" customHeight="1">
-      <c r="E14" s="9" t="s">
-        <v>31</v>
+      <c r="E14" s="6" t="s">
+        <v>29</v>
       </c>
       <c r="F14" s="4"/>
     </row>

</xml_diff>